<commit_message>
Registrar a los ausentes del padrón como falta de esa feria y conservar su puesto
- "Ausente" ya no deja el puesto disponible ni anula el cobro del mes: se guarda una
  falta (F) en asistencias_feriales para la fecha de la feria, que no se cobra; los
  presentes con fecha quedan como P. Al reimportar se actualiza la marca sin duplicar.
- La fecha sale de la columna "Fecha Feria" o de la fecha elegida al subir el archivo;
  debe ser martes o miércoles, y un ausente sin fecha es un error de fila.
- La plantilla oficial suma la columna "Fecha Feria" con validación de día de feria.
- Cliente: selector de fecha de feria junto al archivo (cambiarla vuelve a previsualizar)
  y textos de la importación actualizados.
- Datos de prueba con fechas de feria y dos casos de error nuevos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019to34K7dRuCaHu5NUEVpvW
</commit_message>
<xml_diff>
--- a/datos-prueba/padron-prueba-50.xlsx
+++ b/datos-prueba/padron-prueba-50.xlsx
@@ -17,7 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -60,13 +62,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -445,6 +448,7 @@
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -505,6 +509,11 @@
           <t>Estado</t>
         </is>
       </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Fecha Feria</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -553,6 +562,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K3" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -601,6 +613,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K4" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -649,6 +664,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K5" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -697,6 +715,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K6" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -745,6 +766,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K7" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -793,6 +817,9 @@
           <t>Ausente</t>
         </is>
       </c>
+      <c r="K8" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -841,6 +868,9 @@
           <t>Ausente</t>
         </is>
       </c>
+      <c r="K9" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -889,6 +919,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K10" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -937,6 +970,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K11" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -985,6 +1021,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K12" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1033,6 +1072,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K13" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1081,6 +1123,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K14" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1129,6 +1174,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K15" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1177,6 +1225,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K16" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1225,6 +1276,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K17" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1273,6 +1327,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K18" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1321,6 +1378,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K19" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1369,6 +1429,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K20" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1417,6 +1480,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K21" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1465,6 +1531,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K22" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1513,6 +1582,9 @@
           <t>Ausente</t>
         </is>
       </c>
+      <c r="K23" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1561,6 +1633,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K24" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1609,6 +1684,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K25" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1657,6 +1735,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K26" s="4" t="n">
+        <v>46315</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1704,6 +1785,9 @@
         <is>
           <t>Presente</t>
         </is>
+      </c>
+      <c r="K27" s="4" t="n">
+        <v>46315</v>
       </c>
     </row>
   </sheetData>
@@ -1717,7 +1801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1730,6 +1814,7 @@
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1790,6 +1875,11 @@
           <t>Estado</t>
         </is>
       </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Fecha Feria</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1838,6 +1928,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K3" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1886,6 +1979,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K4" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1934,6 +2030,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K5" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1982,6 +2081,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K6" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -2030,6 +2132,9 @@
           <t>Ausente</t>
         </is>
       </c>
+      <c r="K7" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -2078,6 +2183,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K8" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -2126,6 +2234,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K9" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -2174,6 +2285,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K10" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -2222,6 +2336,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K11" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2270,6 +2387,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K12" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -2318,6 +2438,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K13" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -2366,6 +2489,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K14" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2414,6 +2540,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K15" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2462,6 +2591,9 @@
           <t>Ausente</t>
         </is>
       </c>
+      <c r="K16" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2510,6 +2642,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K17" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2558,6 +2693,9 @@
           <t>Ausente</t>
         </is>
       </c>
+      <c r="K18" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2606,6 +2744,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K19" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -2654,6 +2795,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K20" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -2702,6 +2846,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K21" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2750,6 +2897,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K22" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2798,6 +2948,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K23" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2846,6 +2999,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K24" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2894,6 +3050,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K25" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2942,6 +3101,9 @@
           <t>Presente</t>
         </is>
       </c>
+      <c r="K26" s="4" t="n">
+        <v>46316</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2989,6 +3151,9 @@
         <is>
           <t>Presente</t>
         </is>
+      </c>
+      <c r="K27" s="4" t="n">
+        <v>46316</v>
       </c>
     </row>
   </sheetData>

</xml_diff>